<commit_message>
Some update in Testcasees
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/ElectricCars.xlsx
+++ b/src/test/resources/testData/ElectricCars.xlsx
@@ -104,15 +104,6 @@
     <t>EMI : ₹41,571</t>
   </si>
   <si>
-    <t>Tata Tiago EV</t>
-  </si>
-  <si>
-    <t>₹ 7.99 Lakh</t>
-  </si>
-  <si>
-    <t>EMI : ₹15,456</t>
-  </si>
-  <si>
     <t>Kia EV6</t>
   </si>
   <si>
@@ -131,6 +122,15 @@
     <t>EMI : ₹42,345</t>
   </si>
   <si>
+    <t>VinFast VF MPV 7</t>
+  </si>
+  <si>
+    <t>₹ 24.49 Lakh</t>
+  </si>
+  <si>
+    <t>EMI : ₹47,375</t>
+  </si>
+  <si>
     <t>Vayve Mobility Eva</t>
   </si>
   <si>
@@ -140,13 +140,22 @@
     <t>EMI : ₹6,287</t>
   </si>
   <si>
-    <t>VinFast VF MPV 7</t>
-  </si>
-  <si>
-    <t>₹ 24.49 Lakh</t>
-  </si>
-  <si>
-    <t>EMI : ₹47,375</t>
+    <t>MG ZS EV</t>
+  </si>
+  <si>
+    <t>₹ 17.99 Lakh</t>
+  </si>
+  <si>
+    <t>EMI : ₹34,801</t>
+  </si>
+  <si>
+    <t>Tata Curvv EV</t>
+  </si>
+  <si>
+    <t>₹ 17.49 Lakh</t>
+  </si>
+  <si>
+    <t>EMI : ₹33,834</t>
   </si>
   <si>
     <t>VinFast VF6</t>
@@ -158,24 +167,6 @@
     <t>EMI : ₹33,447</t>
   </si>
   <si>
-    <t>Tata Curvv EV</t>
-  </si>
-  <si>
-    <t>₹ 17.49 Lakh</t>
-  </si>
-  <si>
-    <t>EMI : ₹33,834</t>
-  </si>
-  <si>
-    <t>MG ZS EV</t>
-  </si>
-  <si>
-    <t>₹ 17.99 Lakh</t>
-  </si>
-  <si>
-    <t>EMI : ₹34,801</t>
-  </si>
-  <si>
     <t>Hyundai Creta Electric</t>
   </si>
   <si>
@@ -201,6 +192,15 @@
   </si>
   <si>
     <t>EMI : ₹1.16 Lakh</t>
+  </si>
+  <si>
+    <t>BYD Atto 3</t>
+  </si>
+  <si>
+    <t>₹ 24.99 Lakh</t>
+  </si>
+  <si>
+    <t>EMI : ₹48,342</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added ScreenshotUtil methods in TC_6 and TC_10
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/ElectricCars.xlsx
+++ b/src/test/resources/testData/ElectricCars.xlsx
@@ -50,15 +50,6 @@
     <t>EMI : ₹18,745</t>
   </si>
   <si>
-    <t>MG Windsor EV</t>
-  </si>
-  <si>
-    <t>₹ 14.00 Lakh</t>
-  </si>
-  <si>
-    <t>EMI : ₹27,078</t>
-  </si>
-  <si>
     <t>Mahindra XEV 9e</t>
   </si>
   <si>
@@ -167,6 +158,15 @@
     <t>EMI : ₹33,447</t>
   </si>
   <si>
+    <t>BMW iX1</t>
+  </si>
+  <si>
+    <t>₹ 50.90 Lakh</t>
+  </si>
+  <si>
+    <t>EMI : ₹98,464</t>
+  </si>
+  <si>
     <t>Hyundai Creta Electric</t>
   </si>
   <si>
@@ -176,15 +176,6 @@
     <t>EMI : ₹34,863</t>
   </si>
   <si>
-    <t>BMW iX1</t>
-  </si>
-  <si>
-    <t>₹ 50.90 Lakh</t>
-  </si>
-  <si>
-    <t>EMI : ₹98,464</t>
-  </si>
-  <si>
     <t>Tesla Model Y</t>
   </si>
   <si>
@@ -201,6 +192,15 @@
   </si>
   <si>
     <t>EMI : ₹48,342</t>
+  </si>
+  <si>
+    <t>BMW i7</t>
+  </si>
+  <si>
+    <t>₹ 2.05 Crore</t>
+  </si>
+  <si>
+    <t>EMI : ₹3.97 Lakh</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Some changes in the structure of framework
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/ElectricCars.xlsx
+++ b/src/test/resources/testData/ElectricCars.xlsx
@@ -59,6 +59,15 @@
     <t>EMI : ₹42,364</t>
   </si>
   <si>
+    <t>MG Cyberster</t>
+  </si>
+  <si>
+    <t>₹ 75.00 Lakh</t>
+  </si>
+  <si>
+    <t>EMI : ₹1.45 Lakh</t>
+  </si>
+  <si>
     <t>MG Comet EV</t>
   </si>
   <si>
@@ -68,15 +77,6 @@
     <t>EMI : ₹14,505</t>
   </si>
   <si>
-    <t>MG Cyberster</t>
-  </si>
-  <si>
-    <t>₹ 75.00 Lakh</t>
-  </si>
-  <si>
-    <t>EMI : ₹1.45 Lakh</t>
-  </si>
-  <si>
     <t>Tata Nexon EV</t>
   </si>
   <si>
@@ -131,6 +131,15 @@
     <t>EMI : ₹6,287</t>
   </si>
   <si>
+    <t>Tata Curvv EV</t>
+  </si>
+  <si>
+    <t>₹ 17.49 Lakh</t>
+  </si>
+  <si>
+    <t>EMI : ₹33,834</t>
+  </si>
+  <si>
     <t>MG ZS EV</t>
   </si>
   <si>
@@ -138,15 +147,6 @@
   </si>
   <si>
     <t>EMI : ₹34,801</t>
-  </si>
-  <si>
-    <t>Tata Curvv EV</t>
-  </si>
-  <si>
-    <t>₹ 17.49 Lakh</t>
-  </si>
-  <si>
-    <t>EMI : ₹33,834</t>
   </si>
   <si>
     <t>VinFast VF6</t>

</xml_diff>